<commit_message>
feat: setup UI frontend WMS untuk Sprint 1 sampai 5
</commit_message>
<xml_diff>
--- a/Blueprint Pengerjaan Frontend WMS SaaS.xlsx
+++ b/Blueprint Pengerjaan Frontend WMS SaaS.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="79">
   <si>
     <t>Tahap</t>
   </si>
@@ -52,139 +52,142 @@
     <t>Konfigurasi Zustand (State) &amp; TanStack Query (Data Fetching).</t>
   </si>
   <si>
+    <t>Setup Toast Notifications (Notifikasi Sukses/Gagal).</t>
+  </si>
+  <si>
+    <t>SPRINT 2</t>
+  </si>
+  <si>
+    <t>Auth &amp; Onboarding</t>
+  </si>
+  <si>
+    <t>Buat UI Landing Page (opsional/halaman jualan).</t>
+  </si>
+  <si>
+    <t>Buat halaman Login &amp; Register (/auth/login).</t>
+  </si>
+  <si>
+    <t>API NextAuth / JWT</t>
+  </si>
+  <si>
+    <t>🔐 Alur Auth</t>
+  </si>
+  <si>
+    <t>Buat halaman Onboarding Tenant (Setup nama gudang pertama).</t>
+  </si>
+  <si>
+    <t>POST /api/warehouses</t>
+  </si>
+  <si>
+    <t>🔐 Gateway SaaS</t>
+  </si>
+  <si>
+    <t>SPRINT 3</t>
+  </si>
+  <si>
+    <t>Global Layout</t>
+  </si>
+  <si>
+    <t>Buat Sidebar Navigation yang bisa di-collapse.</t>
+  </si>
+  <si>
+    <t>📱 Responsivitas</t>
+  </si>
+  <si>
+    <t>Buat Top Navbar (Search, Tenant Badge, Profile).</t>
+  </si>
+  <si>
+    <t>Setup Skeleton Loading global &amp; halaman Error 404/500.</t>
+  </si>
+  <si>
+    <t>⏳ Skeleton Loading</t>
+  </si>
+  <si>
+    <t>SPRINT 4</t>
+  </si>
+  <si>
+    <t>Master Data UI</t>
+  </si>
+  <si>
+    <t>UI Tabel Produk dengan Server-side Pagination &amp; Filter.</t>
+  </si>
+  <si>
+    <t>GET/POST /api/products</t>
+  </si>
+  <si>
+    <t>🔍 Pagination &amp; Filter</t>
+  </si>
+  <si>
+    <t>UI Form Tambah Produk (Support Barcode Scanner Input).</t>
+  </si>
+  <si>
+    <t>POST /api/products</t>
+  </si>
+  <si>
+    <t>📱 Mode Scanner</t>
+  </si>
+  <si>
+    <t>UI Manajemen Gudang &amp; Ilustrasi Empty State.</t>
+  </si>
+  <si>
+    <t>GET /api/warehouses</t>
+  </si>
+  <si>
+    <t>⏳ Empty States</t>
+  </si>
+  <si>
+    <t>UI Generate Lokasi Rak/Bin secara massal.</t>
+  </si>
+  <si>
+    <t>GET/POST /api/locations</t>
+  </si>
+  <si>
+    <t>Desain Printable untuk Label Barcode Rak/Produk.</t>
+  </si>
+  <si>
+    <t>🖨️ Printable Layouts</t>
+  </si>
+  <si>
+    <t>SPRINT 5</t>
+  </si>
+  <si>
+    <t>Inbound UI</t>
+  </si>
+  <si>
+    <t>UI Form Receiving (Penerimaan dari Supplier).</t>
+  </si>
+  <si>
+    <t>POST /api/v1/receiving</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>UI Put-away (Tampilan khusus Tablet/PDA untuk Operator).</t>
+  </si>
+  <si>
+    <t>POST /api/v1/put-away</t>
+  </si>
+  <si>
+    <t>📱 Mode Tablet</t>
+  </si>
+  <si>
+    <t>SPRINT 6</t>
+  </si>
+  <si>
+    <t>Inventory UI</t>
+  </si>
+  <si>
+    <t>UI Tabel Stok Real-time (Advanced Filter per Rak/Zone).</t>
+  </si>
+  <si>
+    <t>GET /api/v1/storage/stock</t>
+  </si>
+  <si>
+    <t>🔍 Advanced Filtering</t>
+  </si>
+  <si>
     <t>⬜ To Do</t>
-  </si>
-  <si>
-    <t>Setup Toast Notifications (Notifikasi Sukses/Gagal).</t>
-  </si>
-  <si>
-    <t>SPRINT 2</t>
-  </si>
-  <si>
-    <t>Auth &amp; Onboarding</t>
-  </si>
-  <si>
-    <t>Buat UI Landing Page (opsional/halaman jualan).</t>
-  </si>
-  <si>
-    <t>Buat halaman Login &amp; Register (/auth/login).</t>
-  </si>
-  <si>
-    <t>API NextAuth / JWT</t>
-  </si>
-  <si>
-    <t>🔐 Alur Auth</t>
-  </si>
-  <si>
-    <t>Buat halaman Onboarding Tenant (Setup nama gudang pertama).</t>
-  </si>
-  <si>
-    <t>POST /api/warehouses</t>
-  </si>
-  <si>
-    <t>🔐 Gateway SaaS</t>
-  </si>
-  <si>
-    <t>SPRINT 3</t>
-  </si>
-  <si>
-    <t>Global Layout</t>
-  </si>
-  <si>
-    <t>Buat Sidebar Navigation yang bisa di-collapse.</t>
-  </si>
-  <si>
-    <t>📱 Responsivitas</t>
-  </si>
-  <si>
-    <t>Buat Top Navbar (Search, Tenant Badge, Profile).</t>
-  </si>
-  <si>
-    <t>Setup Skeleton Loading global &amp; halaman Error 404/500.</t>
-  </si>
-  <si>
-    <t>⏳ Skeleton Loading</t>
-  </si>
-  <si>
-    <t>SPRINT 4</t>
-  </si>
-  <si>
-    <t>Master Data UI</t>
-  </si>
-  <si>
-    <t>UI Tabel Produk dengan Server-side Pagination &amp; Filter.</t>
-  </si>
-  <si>
-    <t>GET/POST /api/products</t>
-  </si>
-  <si>
-    <t>🔍 Pagination &amp; Filter</t>
-  </si>
-  <si>
-    <t>UI Form Tambah Produk (Support Barcode Scanner Input).</t>
-  </si>
-  <si>
-    <t>POST /api/products</t>
-  </si>
-  <si>
-    <t>📱 Mode Scanner</t>
-  </si>
-  <si>
-    <t>UI Manajemen Gudang &amp; Ilustrasi Empty State.</t>
-  </si>
-  <si>
-    <t>GET /api/warehouses</t>
-  </si>
-  <si>
-    <t>⏳ Empty States</t>
-  </si>
-  <si>
-    <t>UI Generate Lokasi Rak/Bin secara massal.</t>
-  </si>
-  <si>
-    <t>GET/POST /api/locations</t>
-  </si>
-  <si>
-    <t>Desain Printable untuk Label Barcode Rak/Produk.</t>
-  </si>
-  <si>
-    <t>🖨️ Printable Layouts</t>
-  </si>
-  <si>
-    <t>SPRINT 5</t>
-  </si>
-  <si>
-    <t>Inbound UI</t>
-  </si>
-  <si>
-    <t>UI Form Receiving (Penerimaan dari Supplier).</t>
-  </si>
-  <si>
-    <t>POST /api/v1/receiving</t>
-  </si>
-  <si>
-    <t>UI Put-away (Tampilan khusus Tablet/PDA untuk Operator).</t>
-  </si>
-  <si>
-    <t>POST /api/v1/put-away</t>
-  </si>
-  <si>
-    <t>📱 Mode Tablet</t>
-  </si>
-  <si>
-    <t>SPRINT 6</t>
-  </si>
-  <si>
-    <t>Inventory UI</t>
-  </si>
-  <si>
-    <t>UI Tabel Stok Real-time (Advanced Filter per Rak/Zone).</t>
-  </si>
-  <si>
-    <t>GET /api/v1/storage/stock</t>
-  </si>
-  <si>
-    <t>🔍 Advanced Filtering</t>
   </si>
   <si>
     <t>UI Stock Opname (Form input aktual fisik vs sistem).</t>
@@ -297,13 +300,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -610,12 +616,12 @@
   <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="3" width="32.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -658,7 +664,7 @@
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="21">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -674,11 +680,9 @@
       <c r="E3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="F3" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="21">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -686,264 +690,240 @@
         <v>7</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="21">
+      <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="21">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="1" t="s">
+      <c r="D6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="21">
+      <c r="A7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="21">
+      <c r="A8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="1" t="s">
+      <c r="B8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="F8" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="C9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="21">
+      <c r="A10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="21">
+      <c r="A11" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="1" t="s">
+      <c r="B11" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="D11" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="21">
+      <c r="A12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="1" t="s">
+      <c r="D12" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="21">
+      <c r="A13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" s="1" t="s">
+      <c r="C13" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C13" s="1" t="s">
+      <c r="D13" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="F13" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="C14" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="E14" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="21">
+      <c r="A15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E15" s="1" t="s">
+      <c r="F15" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="21">
+      <c r="A16" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F15" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="1" t="s">
+      <c r="B16" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="D16" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="E16" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="21">
       <c r="A17" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>46</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>49</v>
@@ -955,10 +935,10 @@
         <v>51</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
+        <v>10</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="21">
       <c r="A18" s="1" t="s">
         <v>52</v>
       </c>
@@ -975,7 +955,7 @@
         <v>56</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
@@ -986,16 +966,16 @@
         <v>53</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>12</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
@@ -1006,156 +986,156 @@
         <v>53</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>9</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
       <c r="A22" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>51</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
       <c r="A23" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>9</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
       <c r="A24" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>9</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
       <c r="A27" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>